<commit_message>
docs: add db schema and test codes
</commit_message>
<xml_diff>
--- a/docs/database/data_dictionary.xlsx
+++ b/docs/database/data_dictionary.xlsx
@@ -99,12 +99,12 @@
       </c>
       <c r="I1" t="inlineStr" s="1">
         <is>
-          <t>column_description_ko</t>
+          <t>column_description_en</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>table_description_ko</t>
+          <t>table_description_en</t>
         </is>
       </c>
     </row>
@@ -151,12 +151,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>연결된 운영 위치의 내부 식별자</t>
+          <t>Identifier of the related location.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -203,12 +203,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>위치 계층에서 바로 상위에 있는 운영 위치 식별자</t>
+          <t>Identifier of the related parent location.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -255,12 +255,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>운영 화면과 외부 연동에서 사용하는 위치 고유 코드</t>
+          <t>Business code for location.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -307,12 +307,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>운영자 화면에 표시할 위치 이름</t>
+          <t>Location name displayed in operator interfaces.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -359,12 +359,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>랙, 슬롯, waypoint, 도크, 충전기, 작업장 등 위치 종류 코드</t>
+          <t>Code identifying the location type.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -411,12 +411,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>창고 운영 구역을 식별하는 코드</t>
+          <t>Business code for zone.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -463,12 +463,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>상온 ambient, 냉장 chilled 또는 냉동 frozen 보관 구역 코드</t>
+          <t>Temperature zone for this record.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -515,12 +515,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Open-RMF와 로봇 navigation에서 사용하는 지도 이름</t>
+          <t>Name of the map.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -567,12 +567,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Open-RMF navigation graph의 waypoint 이름</t>
+          <t>Name of the rmf waypoint.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -619,12 +619,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>지도 좌표계 기준 X 좌표이며 단위는 m</t>
+          <t>X coordinate in the map frame, in meters.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -671,12 +671,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>지도 좌표계 기준 Y 좌표이며 단위는 m</t>
+          <t>Y coordinate in the map frame, in meters.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -723,12 +723,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>지도 좌표계 기준 회전각이며 단위는 rad</t>
+          <t>Heading in the map frame, in radians.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -775,12 +775,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>위치의 현재 운영 상태이며 available, reserved, occupied, blocked, maintenance 중 하나</t>
+          <t>Current location status: available, reserved, occupied, blocked, or maintenance.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -827,12 +827,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>위치별 확장 속성과 외부 연동 값을 저장하는 JSON 객체</t>
+          <t>JSON object containing location-specific attributes and external integration values.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>창고의 랙, 슬롯, 도크, 충전기, 작업장, 안전 노드와 RMF waypoint를 통합 관리한다.</t>
+          <t>Manages warehouse racks, slots, docks, chargers, workstations, safety nodes, and RMF waypoints.</t>
         </is>
       </c>
     </row>
@@ -879,12 +879,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>지도 feature를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related feature.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -931,12 +931,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Open-RMF와 로봇 navigation에서 사용하는 지도 이름</t>
+          <t>Name of the map.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>좌표와 feature가 유효한 지도 버전 식별자</t>
+          <t>Map revision for this record.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -1035,12 +1035,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>지도 revision 안에서 feature를 식별하는 업무 코드</t>
+          <t>Business code for feature.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -1087,12 +1087,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>표식, 정적 장애물, 병목, 출입문 또는 진입 금지 구역 코드</t>
+          <t>Code identifying the feature type.</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>연결된 운영 위치의 내부 식별자</t>
+          <t>Identifier of the related location.</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -1191,12 +1191,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>QR 또는 ArUco 표식에서 읽는 숫자 코드</t>
+          <t>Business code for marker.</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -1243,12 +1243,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>지도 좌표계의 점, 선 또는 다각형 공간 정보를 담은 JSON 객체</t>
+          <t>JSON geometry describing a point, line, or polygon in map coordinates.</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -1295,12 +1295,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>지도 feature의 운영 규칙과 표시 속성을 담은 JSON 객체</t>
+          <t>JSON object containing additional properties data.</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>해당 지도 revision에서 feature를 운영 규칙에 사용할지 나타내는 값</t>
+          <t>Indicates whether this feature is used by operating rules for the map revision.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>지도 revision별 표식, 정적 장애물, 병목, 출입문과 진입 금지 구역의 공간 정보를 관리한다.</t>
+          <t>Manages spatial data for markers, static obstacles, bottlenecks, doors, and restricted areas by map revision.</t>
         </is>
       </c>
     </row>
@@ -1399,12 +1399,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>작업자 계정을 식별하는 내부 고유 값</t>
+          <t>Identifier of the related worker.</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1451,12 +1451,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>운영 화면과 인증 연동에서 사용하는 작업자 고유 코드</t>
+          <t>Business code for worker.</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1503,12 +1503,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>운영자 화면과 감사 기록에 표시할 작업자 이름</t>
+          <t>Worker name displayed in operator interfaces and audit records.</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1555,12 +1555,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>작업자의 운영 권한 역할 코드</t>
+          <t>Role for this record.</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1607,12 +1607,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>SSO 또는 외부 인증 시스템에서 사용하는 작업자 식별자</t>
+          <t>Identifier of the related external auth.</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1659,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>작업자가 접근하거나 조작할 수 있는 구역 코드의 JSON 배열</t>
+          <t>JSON array of zone codes the worker may access or operate.</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1711,12 +1711,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>작업자 계정이 현재 업무 요청과 승인에 참여할 수 있는지 나타내는 값</t>
+          <t>Indicates whether this worker account may participate in job requests and approvals.</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1763,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>작업자 또는 장비가 운영 시스템에 등록된 시각</t>
+          <t>Timestamp when the registered event occurred.</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1815,12 +1815,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>작업자 또는 장비를 운영 대상에서 제외한 시각</t>
+          <t>Timestamp when the retired event occurred.</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>관제 요청, 수동 복구와 안전 해제에 대한 책임을 식별할 작업자 계정과 권한 범위를 관리한다.</t>
+          <t>Manages worker accounts and permission scopes for control requests, manual recovery, and safety release actions.</t>
         </is>
       </c>
     </row>
@@ -1867,12 +1867,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Pinky 또는 OMX 장비를 식별하는 고유 코드</t>
+          <t>Identifier of the related device.</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>장비를 주행로봇 mobile 또는 로봇팔 arm으로 구분하는 코드</t>
+          <t>Code identifying the device type.</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -1971,12 +1971,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>운영자 화면에 표시할 장비 이름</t>
+          <t>Device name displayed in operator interfaces.</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2023,12 +2023,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>장비 제조사 또는 제품 모델 이름</t>
+          <t>Model for this record.</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2075,12 +2075,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>주행로봇이 소속된 Open-RMF fleet 이름</t>
+          <t>Name of the fleet.</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2127,12 +2127,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>장비가 대기하거나 복귀할 기본 운영 위치 식별자</t>
+          <t>Identifier of the related home location.</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2179,12 +2179,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>장비가 현재 위치한 것으로 확정된 운영 위치 식별자</t>
+          <t>Identifier of the related current location.</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2231,12 +2231,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>장비의 자동, 수동, 오프라인, 정비 또는 안전 정지 제어 모드</t>
+          <t>Device control mode, such as automatic, manual, offline, maintenance, or safety stop.</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2283,12 +2283,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>장비가 현재 배차와 작업 할당 대상인지 나타내는 값</t>
+          <t>Indicates whether this device is eligible for dispatch and job assignment.</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2335,12 +2335,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>장비가 지원하는 동작과 기능을 표현한 JSON 객체</t>
+          <t>JSON object describing actions and features supported by the device.</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2387,12 +2387,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>작업자 또는 장비가 운영 시스템에 등록된 시각</t>
+          <t>Timestamp when the registered event occurred.</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2439,12 +2439,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>작업자 또는 장비를 운영 대상에서 제외한 시각</t>
+          <t>Timestamp when the retired event occurred.</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Pinky 주행로봇과 OMX 로봇팔의 모델, 소속, 위치, 제어 모드와 기능을 관리한다.</t>
+          <t>Manages models, fleets, locations, control modes, and capabilities for Pinky mobile robots and OMX robot arms.</t>
         </is>
       </c>
     </row>
@@ -2491,12 +2491,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>연결된 재고 로트의 내부 식별자</t>
+          <t>Identifier of the related lot.</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2543,12 +2543,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>상품 종류를 식별하는 업무 코드</t>
+          <t>Business code for product.</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2595,12 +2595,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>입고 단위와 추적에 사용하는 재고 로트 고유 코드</t>
+          <t>Business code for lot.</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2647,12 +2647,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>운영자 화면에 표시할 상품 이름</t>
+          <t>Name of the item.</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>상온 ambient, 냉장 chilled 또는 냉동 frozen 보관 구역 코드</t>
+          <t>Temperature zone for this record.</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2751,12 +2751,12 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>연결된 운영 위치의 내부 식별자</t>
+          <t>Identifier of the related location.</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2803,12 +2803,12 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>재고 로트의 유통기한 날짜</t>
+          <t>Expiry date for this record.</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2855,12 +2855,12 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>상품 한 단위의 kg 기준 무게</t>
+          <t>Weight of one product unit in kilograms.</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2907,12 +2907,12 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>현재 로트에서 물리적으로 보유한 전체 수량</t>
+          <t>Total physical quantity currently held in the inventory lot.</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -2959,12 +2959,12 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>출고 등의 업무를 위해 선점된 수량</t>
+          <t>Quantity for reserved.</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -3011,12 +3011,12 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>재고 로트의 입고 대기, 보관, 보류, 소진, 만료 또는 손상 상태</t>
+          <t>Inventory-lot status, such as pending receipt, stored, held, depleted, expired, or damaged.</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -3063,12 +3063,12 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>재고 로트의 입고가 완료된 시각</t>
+          <t>Timestamp when the received event occurred.</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -3115,12 +3115,12 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>해당 레코드가 마지막으로 수정된 시각</t>
+          <t>Timestamp when the updated event occurred.</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>상품 로트별 보관 위치, 유통기한, 가용 수량, 예약 수량과 보관 상태를 관리한다.</t>
+          <t>Manages storage location, expiration date, available quantity, reserved quantity, and status for each inventory lot.</t>
         </is>
       </c>
     </row>
@@ -3167,12 +3167,12 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>업무를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job.</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3219,12 +3219,12 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>하위 업무를 생성한 상위 업무의 식별자</t>
+          <t>Identifier of the related parent job.</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>운영 화면과 외부 연동에서 사용하는 업무 고유 코드</t>
+          <t>Business code for job.</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3323,12 +3323,12 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구 또는 비상 업무 종류 코드</t>
+          <t>Code identifying the operation type.</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3375,12 +3375,12 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>업무의 critical, high, normal 또는 low 우선순위 코드</t>
+          <t>Job priority code: critical, high, normal, or low.</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3427,12 +3427,12 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>우선순위 정렬을 위해 자동 계산되는 숫자 값</t>
+          <t>Automatically calculated numeric value used to sort priorities.</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>업무의 대기부터 계획, 실행, 완료, 실패, 취소와 안전 보류까지의 상태</t>
+          <t>Job lifecycle status from pending and planning through execution, completion, failure, cancellation, or safety hold.</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3531,12 +3531,12 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>동시 수정 충돌을 탐지하기 위한 낙관적 잠금 버전</t>
+          <t>Optimistic-lock version used to detect concurrent updates.</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3583,12 +3583,12 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>업무 생성을 요청한 작업자의 식별자</t>
+          <t>Requested by for this record.</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3635,12 +3635,12 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>외부 시스템의 요청이나 작업과 연결하는 참조 값</t>
+          <t>External reference for this record.</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3687,12 +3687,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>업무가 시작되는 운영 위치 식별자</t>
+          <t>Identifier of the related source location.</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3739,12 +3739,12 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>업무가 최종적으로 도착해야 하는 운영 위치 식별자</t>
+          <t>Identifier of the related destination location.</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3791,12 +3791,12 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>업무 완료가 요구되는 기한 시각</t>
+          <t>Timestamp when the due event occurred.</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3843,12 +3843,12 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>업무에 배정된 Pinky 주행로봇의 장비 식별자</t>
+          <t>Identifier of the related assigned mobile.</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3895,12 +3895,12 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>업무 또는 실행 단계가 실패한 구체적인 원인</t>
+          <t>Specific reason the job or execution step failed.</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3947,12 +3947,12 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>업무 생성 원인과 외부 요청의 확장 맥락을 저장하는 JSON 객체</t>
+          <t>JSON object containing the job origin and extended context from external requests.</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -3999,12 +3999,12 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>해당 레코드가 데이터베이스에 생성된 시각</t>
+          <t>Timestamp when the created event occurred.</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -4051,12 +4051,12 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>업무, 단계 또는 복구 행동이 실제로 시작된 시각</t>
+          <t>Timestamp when the started event occurred.</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -4103,12 +4103,12 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>업무, 단계 또는 복구 행동이 완료된 시각</t>
+          <t>Timestamp when the completed event occurred.</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>입고, 출고, 이동, 보충, 폐기, 복구와 비상 대응 업무의 전체 수명주기를 관리한다.</t>
+          <t>Manages the full lifecycle of inbound, outbound, transfer, replenishment, disposal, recovery, and emergency jobs.</t>
         </is>
       </c>
     </row>
@@ -4155,12 +4155,12 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>업무 품목을 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job item.</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4207,12 +4207,12 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>업무를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job.</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4259,12 +4259,12 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>상품 종류를 식별하는 업무 코드</t>
+          <t>Business code for product.</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4311,12 +4311,12 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>업무에서 처리하도록 요청한 상품 수량</t>
+          <t>Quantity for requested.</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4363,12 +4363,12 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>업무 품목 중 실제 처리가 완료된 수량</t>
+          <t>Quantity for completed.</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4415,12 +4415,12 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>연결된 재고 로트의 내부 식별자</t>
+          <t>Identifier of the related lot.</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4467,12 +4467,12 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>바구니, 박스 또는 팔레트 등 취급 단위의 식별 코드</t>
+          <t>Business code for handling unit.</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4519,12 +4519,12 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>업무 품목의 미검수, 일치, 불일치 또는 수동 검토 상태 코드</t>
+          <t>Verification state for this record.</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4571,12 +4571,12 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>업무 품목별 검수와 외부 주문의 확장 값을 저장하는 JSON 객체</t>
+          <t>JSON object containing item-specific verification and external-order values.</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>업무에 포함된 상품, 요청 수량, 완료 수량, 배정 로트와 검수 상태를 관리한다.</t>
+          <t>Manages products, requested and completed quantities, assigned lots, and verification status for each job.</t>
         </is>
       </c>
     </row>
@@ -4623,12 +4623,12 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>업무 실행 단계를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job step.</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -4675,12 +4675,12 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>업무를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job.</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -4727,12 +4727,12 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>같은 업무 또는 에피소드 안에서 실행 순서를 나타내는 번호</t>
+          <t>Execution order within the same job or recovery episode.</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -4779,12 +4779,12 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>업무 단계의 실행 주체를 mobile, arm 또는 fms로 구분하는 코드</t>
+          <t>Code identifying the executor type.</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -4831,12 +4831,12 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>업무 단계를 실행하도록 배정된 장비 식별자</t>
+          <t>Identifier of the related assigned device.</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -4883,12 +4883,12 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>실행할 동작 종류를 나타내는 코드 값</t>
+          <t>Code identifying the action type.</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -4935,12 +4935,12 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>업무 단계가 이동하거나 조작할 목표 운영 위치 식별자</t>
+          <t>Identifier of the related target location.</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -4987,12 +4987,12 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>업무 단계의 대기, 큐 등록, 실행, 성공, 실패, 보류 또는 취소 상태</t>
+          <t>Job-step status: pending, queued, running, succeeded, failed, held, or cancelled.</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5039,12 +5039,12 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Open-RMF에서 발급한 이동 작업 식별자</t>
+          <t>Identifier of the related rmf task.</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5091,12 +5091,12 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>업무 단계 판단에 사용한 정책 이름</t>
+          <t>Name of the policy.</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5143,12 +5143,12 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>업무 단계 판단에 사용한 정책 버전</t>
+          <t>Policy version for this record.</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5195,12 +5195,12 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>업무 단계 실행을 다시 시도한 누적 횟수</t>
+          <t>Total number of retries for this job step.</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5247,12 +5247,12 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>업무 또는 실행 단계가 실패한 구체적인 원인</t>
+          <t>Specific reason the job or execution step failed.</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>업무 단계를 실행할 때 전달한 입력 값을 저장하는 JSON 객체</t>
+          <t>JSON object containing additional input data.</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5351,12 +5351,12 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>업무 단계 실행 후 반환된 결과를 저장하는 JSON 객체</t>
+          <t>JSON object containing additional result data.</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5403,12 +5403,12 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>업무, 단계 또는 복구 행동이 실제로 시작된 시각</t>
+          <t>Timestamp when the started event occurred.</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5455,12 +5455,12 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>업무, 단계 또는 복구 행동이 완료된 시각</t>
+          <t>Timestamp when the completed event occurred.</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>업무를 Pinky 이동, OMX 조작, 검수와 인계 단위의 순서 있는 실행 단계로 관리한다.</t>
+          <t>Manages ordered execution steps for Pinky movement, OMX manipulation, verification, and handoff operations.</t>
         </is>
       </c>
     </row>
@@ -5507,12 +5507,12 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>자원 예약을 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related reservation.</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5559,12 +5559,12 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>업무를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job.</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5611,12 +5611,12 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>업무 실행 단계를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job step.</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5663,12 +5663,12 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>연결된 운영 위치의 내부 식별자</t>
+          <t>Identifier of the related location.</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5715,12 +5715,12 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Pinky 또는 OMX 장비를 식별하는 고유 코드</t>
+          <t>Identifier of the related device.</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5767,12 +5767,12 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>병목 잠금과 연결된 지도 feature 식별자</t>
+          <t>Identifier of the related map feature.</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5819,12 +5819,12 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>독점 잠금, 병목 잠금 또는 시간 예약 방식 코드</t>
+          <t>Reservation mode for this record.</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5871,12 +5871,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>예약의 reserved, in_use, released, expired 또는 cancelled 상태</t>
+          <t>Reservation status: reserved, in use, released, expired, or cancelled.</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5923,12 +5923,12 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>예약 자원의 사용을 시작할 예정 시각</t>
+          <t>Timestamp when the planned start event occurred.</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -5975,12 +5975,12 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>예약 자원의 사용을 마칠 예정 시각</t>
+          <t>Timestamp when the planned end event occurred.</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -6027,12 +6027,12 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>장비가 예약 자원에 실제로 진입한 시각</t>
+          <t>Timestamp when the entered event occurred.</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -6079,12 +6079,12 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>장비가 예약 자원에서 실제로 빠져나온 시각</t>
+          <t>Timestamp when the exited event occurred.</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -6131,12 +6131,12 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>점유 확인이 없을 때 예약을 자동 만료할 기준 시각</t>
+          <t>Timestamp when the expires event occurred.</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -6183,12 +6183,12 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>해당 레코드가 데이터베이스에 생성된 시각</t>
+          <t>Timestamp when the created event occurred.</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -6235,12 +6235,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>예약 자원이 정상 또는 수동으로 해제된 시각</t>
+          <t>Timestamp when the released event occurred.</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -6287,12 +6287,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>활성 예약의 자원 중복을 방지하기 위해 계산한 고유 키</t>
+          <t>Calculated unique key that prevents conflicting active resource reservations.</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>병목 통로의 진입 권한과 도크, 작업장, 장비의 독점 또는 시간대별 사용 예약을 관리한다.</t>
+          <t>Manages access to bottlenecks and exclusive or time-based reservations for docks, workstations, and devices.</t>
         </is>
       </c>
     </row>
@@ -6339,12 +6339,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>재고 변동 이력을 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related inventory move.</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6391,12 +6391,12 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>연결된 재고 로트의 내부 식별자</t>
+          <t>Identifier of the related lot.</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6443,12 +6443,12 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>업무를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job.</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6495,12 +6495,12 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>업무 실행 단계를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job step.</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6547,12 +6547,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>입고, 출고, 예약, 해제, 조정 등 재고 변동 종류 코드</t>
+          <t>Code identifying the move type.</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6599,12 +6599,12 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>가용 수량에 더하거나 뺀 변화량</t>
+          <t>Amount added to or removed from the available quantity.</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6651,12 +6651,12 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>재고 변동을 반영한 뒤의 가용 수량</t>
+          <t>Available quantity after applying the inventory movement.</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6703,12 +6703,12 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>예약 수량에 더하거나 뺀 변화량</t>
+          <t>Amount added to or removed from the reserved quantity.</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6755,12 +6755,12 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>재고 변동을 반영한 뒤의 예약 수량</t>
+          <t>Reserved quantity after applying the inventory movement.</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6807,12 +6807,12 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>재고 변동을 확정한 서비스 또는 작업자 식별 값</t>
+          <t>Recorded by for this record.</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6859,12 +6859,12 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>재고 변동이 확정되어 기록된 시각</t>
+          <t>Timestamp when the recorded event occurred.</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6911,12 +6911,12 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>재고 변동의 사유를 보충하는 설명</t>
+          <t>Additional explanation for the inventory movement.</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>재고와 예약 수량이 변한 원인, 증감량, 변경 후 수량과 책임 주체를 불변 이력으로 기록한다.</t>
+          <t>Records immutable inventory and reservation quantity changes, resulting balances, reasons, and responsible actors.</t>
         </is>
       </c>
     </row>
@@ -6963,12 +6963,12 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Pinky 또는 OMX 장비를 식별하는 고유 코드</t>
+          <t>Identifier of the related device.</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7015,12 +7015,12 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>장비 상태가 실제로 관측된 시각</t>
+          <t>Timestamp when the observed event occurred.</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7067,12 +7067,12 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>장비가 보고한 현재 동작 상태 코드</t>
+          <t>Current operating-state code reported by the device.</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7119,12 +7119,12 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>장비의 정상, 경고, 오류 또는 통신 두절 건강 상태 코드</t>
+          <t>Device health code, such as healthy, warning, error, or unreachable.</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7171,12 +7171,12 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>장비가 현재 실행 중이라고 보고한 업무 단계 식별자</t>
+          <t>Identifier of the related current job step.</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7223,12 +7223,12 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>지도 좌표계 기준 X 좌표이며 단위는 m</t>
+          <t>X coordinate in the map frame, in meters.</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7275,12 +7275,12 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>지도 좌표계 기준 Y 좌표이며 단위는 m</t>
+          <t>Y coordinate in the map frame, in meters.</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7327,12 +7327,12 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>지도 좌표계 기준 회전각이며 단위는 rad</t>
+          <t>Heading in the map frame, in radians.</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7379,12 +7379,12 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>장비가 보고한 배터리 잔량 백분율</t>
+          <t>Remaining battery percentage reported by the device.</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7431,12 +7431,12 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>현재 업무 단계의 진행률이며 0 이상 1 이하로 저장</t>
+          <t>Progress of the current job step, from 0 through 1.</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7483,12 +7483,12 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>장비별 추가 상태와 진단 값을 저장하는 JSON 객체</t>
+          <t>JSON object containing additional details data.</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>장비별 최신 heartbeat, 위치, 배터리, 진행률, 건강 상태와 현재 실행 단계를 관리한다.</t>
+          <t>Stores the latest heartbeat, location, battery level, progress, health, and active step for each device.</t>
         </is>
       </c>
     </row>
@@ -7535,12 +7535,12 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>시스템 간 메시지를 중복 없이 식별하는 UUID</t>
+          <t>Identifier of the related message.</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -7587,12 +7587,12 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>메시지의 수신 inbound 또는 송신 outbound 방향 코드</t>
+          <t>Message direction: inbound or outbound.</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -7639,12 +7639,12 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>메시지가 통신하는 rmf, pinky 또는 omx 채널 코드</t>
+          <t>Channel for this record.</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -7691,12 +7691,12 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Pinky 또는 OMX 장비를 식별하는 고유 코드</t>
+          <t>Identifier of the related device.</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -7743,12 +7743,12 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>업무 실행 단계를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job step.</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -7795,12 +7795,12 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>명령, 상태 또는 응답의 계약 종류를 나타내는 코드</t>
+          <t>Code identifying the message type.</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -7847,12 +7847,12 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>같은 요청의 중복 실행을 방지하는 업무 멱등 키</t>
+          <t>Business key that prevents duplicate execution of the same request.</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -7899,12 +7899,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>외부 시스템의 요청이나 작업과 연결하는 참조 값</t>
+          <t>External reference for this record.</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -7951,12 +7951,12 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>메시지의 pending, sent, acknowledged, failed 또는 dead 상태</t>
+          <t>Message status: pending, sent, acknowledged, failed, or dead.</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -8003,12 +8003,12 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>메시지 전송을 시도한 누적 횟수</t>
+          <t>Total number of message delivery attempts.</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -8055,12 +8055,12 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>실패한 메시지를 다음에 재전송할 예정 시각</t>
+          <t>Timestamp when the next attempt event occurred.</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -8107,12 +8107,12 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>연동 메시지 또는 운영 이벤트의 원본 데이터를 담은 JSON 객체</t>
+          <t>JSON object containing additional payload data.</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -8159,12 +8159,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>가장 최근 메시지 전송 실패의 원인</t>
+          <t>Last error for this record.</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -8211,12 +8211,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>해당 레코드가 데이터베이스에 생성된 시각</t>
+          <t>Timestamp when the created event occurred.</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -8263,12 +8263,12 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>메시지가 외부 채널로 전송된 시각</t>
+          <t>Timestamp when the sent event occurred.</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -8315,12 +8315,12 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>안전 사건 또는 메시지를 인지했다고 확정한 시각</t>
+          <t>Timestamp when the acknowledged event occurred.</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>RMF, Pinky, OMX와 주고받는 명령과 응답의 멱등 처리, 재전송, 전송 완료 상태를 관리한다.</t>
+          <t>Manages idempotency, retries, and delivery status for commands and responses exchanged with RMF, Pinky, and OMX.</t>
         </is>
       </c>
     </row>
@@ -8367,12 +8367,12 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>안전 사건을 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related incident.</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8419,12 +8419,12 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>운영 화면과 보고서에서 사용하는 안전 사건 고유 코드</t>
+          <t>Business code for incident.</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8471,12 +8471,12 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>사람, 낙상, 충돌 위험, 비상 정지 등 사건 종류 코드</t>
+          <t>Code identifying the incident type.</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8523,12 +8523,12 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>사건 또는 이벤트의 영향 수준을 나타내는 코드</t>
+          <t>Severity for this record.</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8575,12 +8575,12 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>안전 사건의 open, acknowledged, mitigating, resolved 또는 closed 상태</t>
+          <t>Safety-incident status: open, acknowledged, mitigating, resolved, or closed.</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8627,12 +8627,12 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>연결된 운영 위치의 내부 식별자</t>
+          <t>Identifier of the related location.</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8679,12 +8679,12 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>안전 사건이 영향을 주는 점 또는 구역을 표현한 JSON 공간 정보</t>
+          <t>JSON geometry describing the point or area affected by the safety incident.</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8731,12 +8731,12 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>안전 사건의 원인과 상황을 운영자가 이해할 수 있게 기록한 설명</t>
+          <t>Operator-readable description of the cause and circumstances of the safety incident.</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8783,12 +8783,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>안전 사건을 수동으로 등록한 작업자 식별자</t>
+          <t>Identifier of the related raised by worker.</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8835,12 +8835,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>안전 사건을 인지 처리한 작업자의 식별자</t>
+          <t>Identifier of the related acknowledged by worker.</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8887,12 +8887,12 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>안전 사건을 최종 해소 처리한 작업자 식별자</t>
+          <t>Identifier of the related resolved by worker.</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8939,12 +8939,12 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>안전 사건이 최초로 발생하거나 등록된 시각</t>
+          <t>Timestamp when the raised event occurred.</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -8991,12 +8991,12 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>안전 사건 또는 메시지를 인지했다고 확정한 시각</t>
+          <t>Timestamp when the acknowledged event occurred.</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -9043,12 +9043,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>안전 사건의 원인이 제거되어 해소된 시각</t>
+          <t>Timestamp when the resolved event occurred.</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -9095,12 +9095,12 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>센서 관측과 대응 절차 등 안전 사건의 추가 정보를 저장하는 JSON 객체</t>
+          <t>JSON object containing sensor observations, response procedures, and other incident details.</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>사람 감지, 낙상 후보, 충돌 위험, 비상 정지 등 안전 사건의 인지부터 해소까지를 관리한다.</t>
+          <t>Manages safety incidents from detection through resolution, including people, fall risks, collision risks, and emergency stops.</t>
         </is>
       </c>
     </row>
@@ -9147,12 +9147,12 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>운영 이벤트를 내부에서 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related event.</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9199,12 +9199,12 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>시스템 간 중복 없이 운영 이벤트를 식별하는 UUID</t>
+          <t>UUID of the related event.</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9251,12 +9251,12 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>운영 이벤트가 실제로 발생한 시각</t>
+          <t>Timestamp when the occurred event occurred.</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9303,12 +9303,12 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>운영 이벤트의 사용자 조치를 수행한 작업자 식별자</t>
+          <t>Identifier of the related actor worker.</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9355,12 +9355,12 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Pinky 또는 OMX 장비를 식별하는 고유 코드</t>
+          <t>Identifier of the related device.</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9407,12 +9407,12 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>업무를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job.</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9459,12 +9459,12 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>업무 실행 단계를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job step.</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9511,12 +9511,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>안전 사건을 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related incident.</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9563,12 +9563,12 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>사건 또는 이벤트의 영향 수준을 나타내는 코드</t>
+          <t>Severity for this record.</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9615,12 +9615,12 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>운영 이벤트가 속한 기능 영역을 구분하는 코드 값</t>
+          <t>Category for this record.</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9667,12 +9667,12 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>발생한 운영 이벤트의 세부 종류를 나타내는 코드</t>
+          <t>Code identifying the event type.</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9719,12 +9719,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>운영자가 이벤트를 이해할 수 있도록 기록한 요약 메시지</t>
+          <t>Operator-readable summary of the operation event.</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9771,12 +9771,12 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>판단 또는 산출물 생성에 사용한 모델 이름</t>
+          <t>Name of the model.</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9823,12 +9823,12 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>판단 또는 산출물 생성에 사용한 모델 버전</t>
+          <t>Model version for this record.</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9875,12 +9875,12 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>모델 판단의 신뢰도 값이며 0 이상 1 이하로 저장</t>
+          <t>Model confidence value from 0 through 1.</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9927,12 +9927,12 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>모델 제안에 대한 안전 계층의 승인, 거부 또는 보류 결정 코드</t>
+          <t>Safety decision for this record.</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -9979,12 +9979,12 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>이벤트 종류별 상세 관측과 판단 근거를 저장하는 JSON 객체</t>
+          <t>JSON object containing detailed observations and decision evidence for the event type.</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>업무, 장비, 안전, 모델 판단과 운영자 조치의 시간순 감사 이벤트를 기록한다.</t>
+          <t>Records chronological audit events for jobs, devices, safety decisions, model decisions, and operator actions.</t>
         </is>
       </c>
     </row>
@@ -10031,12 +10031,12 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>파일 산출물을 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related artifact.</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10083,12 +10083,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>산출물의 형식을 구분하는 코드 값</t>
+          <t>Code identifying the artifact type.</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10135,12 +10135,12 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>산출물 파일이 보관된 객체 저장소 또는 파일 시스템 URI</t>
+          <t>URI of the stored storage data.</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10187,12 +10187,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>긴 저장 URI의 중복을 검사하기 위해 계산한 이진 해시</t>
+          <t>Storage uri hash for this record.</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10239,12 +10239,12 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>산출물 내용의 무결성을 확인하는 SHA-256 해시</t>
+          <t>SHA-256 hash used to verify the integrity of the sha256.</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10291,12 +10291,12 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>산출물 파일의 MIME 형식</t>
+          <t>Code identifying the mime type.</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10343,12 +10343,12 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>산출물 파일의 바이트 단위 크기</t>
+          <t>Byte size for this record.</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10395,12 +10395,12 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Pinky 또는 OMX 장비를 식별하는 고유 코드</t>
+          <t>Identifier of the related device.</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10447,12 +10447,12 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>업무를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job.</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10499,12 +10499,12 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>업무 실행 단계를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related job step.</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10551,12 +10551,12 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>운영 이벤트를 내부에서 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related event.</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10603,12 +10603,12 @@
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>판단 또는 산출물 생성에 사용한 모델 이름</t>
+          <t>Name of the model.</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10655,12 +10655,12 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>판단 또는 산출물 생성에 사용한 모델 버전</t>
+          <t>Model version for this record.</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10707,12 +10707,12 @@
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>코덱, 해상도, dataset split 등 산출물별 확장 정보를 저장하는 JSON 객체</t>
+          <t>JSON object containing artifact-specific details such as codec, resolution, and dataset split.</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10759,12 +10759,12 @@
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>산출물의 원본 데이터가 취득된 시각</t>
+          <t>Timestamp when the captured event occurred.</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>영상, 이미지, rosbag, episode, dataset, model과 보고서의 저장 위치와 무결성 정보를 관리한다.</t>
+          <t>Manages storage locations and integrity metadata for videos, images, rosbags, episodes, datasets, models, and reports.</t>
         </is>
       </c>
     </row>
@@ -10811,12 +10811,12 @@
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>복구 목표로 사용할 안전 노드를 식별하는 UUID</t>
+          <t>UUID of the related reference node.</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -10863,12 +10863,12 @@
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>연결된 운영 위치의 내부 식별자</t>
+          <t>Identifier of the related location.</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -10915,12 +10915,12 @@
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>좌표와 feature가 유효한 지도 버전 식별자</t>
+          <t>Map revision for this record.</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -10967,12 +10967,12 @@
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>안전 노드가 지원하는 wait, retreat, detour, rejoin 역할의 JSON 배열</t>
+          <t>Recovery roles for this record.</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11019,12 +11019,12 @@
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>복구 기준 노드의 현재 사용 가능 상태 코드</t>
+          <t>Current availability status code.</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11071,12 +11071,12 @@
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>복구 노드 성공 신뢰도의 베타 분포 alpha 누적 값</t>
+          <t>Accumulated beta-distribution alpha value for successful recovery-node outcomes.</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11123,12 +11123,12 @@
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>복구 노드 실패 신뢰도의 베타 분포 beta 누적 값</t>
+          <t>Accumulated beta-distribution beta value for failed recovery-node outcomes.</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11175,12 +11175,12 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>복구 기준 노드의 위치와 안전성을 마지막으로 검증한 시각</t>
+          <t>Timestamp when the last verified event occurred.</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11227,12 +11227,12 @@
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>복구 기준 노드가 실제 결과에 사용된 가장 최근 시각</t>
+          <t>Timestamp when the last outcome event occurred.</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11279,12 +11279,12 @@
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>복구 기준 노드의 상태를 마지막으로 검토한 작업자 식별자</t>
+          <t>Identifier of the related reviewed by worker.</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11331,12 +11331,12 @@
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>동시 수정 충돌을 탐지하기 위한 낙관적 잠금 버전</t>
+          <t>Optimistic-lock version used to detect concurrent updates.</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11383,12 +11383,12 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>복구 기준 노드의 검토 결과와 주의사항</t>
+          <t>Review notes and cautions for the recovery reference node.</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11435,12 +11435,12 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>해당 레코드가 데이터베이스에 생성된 시각</t>
+          <t>Timestamp when the created event occurred.</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11487,12 +11487,12 @@
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>해당 레코드가 마지막으로 수정된 시각</t>
+          <t>Timestamp when the updated event occurred.</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>안전 노드별 복구 역할, 사용 가능 상태와 베타 분포 기반 신뢰도를 관리한다.</t>
+          <t>Manages recovery roles, availability, and beta-distribution reliability values for each safety node.</t>
         </is>
       </c>
     </row>
@@ -11539,12 +11539,12 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>하나의 복구 사건을 시스템 간 고유하게 식별하는 UUID</t>
+          <t>UUID of the related recovery episode.</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -11591,12 +11591,12 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>복구 에피소드를 시작시킨 FMS 운영 이벤트 UUID</t>
+          <t>UUID of the related source event.</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -11643,12 +11643,12 @@
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>Pinky 또는 OMX 장비를 식별하는 고유 코드</t>
+          <t>Identifier of the related device.</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -11695,12 +11695,12 @@
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>복구 에피소드와 연결된 FMS 업무 식별자이며 물리적 외래 키는 두지 않음</t>
+          <t>Identifier of the related fms job.</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -11747,12 +11747,12 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>복구 에피소드와 연결된 FMS 업무 단계 식별자이며 물리적 외래 키는 두지 않음</t>
+          <t>Identifier of the related fms job step.</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -11799,12 +11799,12 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>Open-RMF와 로봇 navigation에서 사용하는 지도 이름</t>
+          <t>Name of the map.</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -11851,12 +11851,12 @@
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>좌표와 feature가 유효한 지도 버전 식별자</t>
+          <t>Map revision for this record.</t>
         </is>
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -11903,12 +11903,12 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>복구를 시작시킨 정체, 사람, 저시정 또는 위치 추정 문제 코드</t>
+          <t>Code identifying the trigger type.</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -11955,12 +11955,12 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>복구 상황 해석에 사용한 VLM 모델 이름</t>
+          <t>Name of the vlm model.</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12007,12 +12007,12 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>복구 상황 해석에 사용한 VLM 모델 버전</t>
+          <t>Vlm model version for this record.</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12059,12 +12059,12 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>실행한 복구 정책의 이름</t>
+          <t>Name of the recovery policy.</t>
         </is>
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12111,12 +12111,12 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>실행한 복구 정책의 버전</t>
+          <t>Recovery policy version for this record.</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12163,12 +12163,12 @@
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>업무, 단계 또는 복구 행동이 실제로 시작된 시각</t>
+          <t>Timestamp when the started event occurred.</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12215,12 +12215,12 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>복구 에피소드가 성공, 중단 또는 실패로 종료된 시각</t>
+          <t>Timestamp when the ended event occurred.</t>
         </is>
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12267,12 +12267,12 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>복구 에피소드의 실행 중, 성공, 중단 또는 실패 최종 상태</t>
+          <t>Current final status code.</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12319,12 +12319,12 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>복구 에피소드의 원인, 행동과 결과를 요약한 설명</t>
+          <t>Summary for this record.</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12371,12 +12371,12 @@
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>해당 레코드가 데이터베이스에 생성된 시각</t>
+          <t>Timestamp when the created event occurred.</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>복구 trigger부터 종료까지 하나의 사건과 사용한 VLM 및 복구 정책의 계보를 기록한다.</t>
+          <t>Records each recovery incident from trigger to completion, including VLM and recovery-policy lineage.</t>
         </is>
       </c>
     </row>
@@ -12423,12 +12423,12 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>복구 실행 단계를 식별하는 자동 증가 번호</t>
+          <t>Identifier of the related recovery step.</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12475,12 +12475,12 @@
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>하나의 복구 사건을 시스템 간 고유하게 식별하는 UUID</t>
+          <t>UUID of the related recovery episode.</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12527,12 +12527,12 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>같은 업무 또는 에피소드 안에서 실행 순서를 나타내는 번호</t>
+          <t>Execution order within the same job or recovery episode.</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12579,12 +12579,12 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>행동 목표로 선택한 FMS 복구 기준 노드 UUID이며 물리적 외래 키는 두지 않음</t>
+          <t>UUID of the FMS recovery reference node selected as the action target; no physical cross-database foreign key is used.</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12631,12 +12631,12 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>실행할 동작 종류를 나타내는 코드 값</t>
+          <t>Code identifying the action type.</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12683,12 +12683,12 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>복구 행동이 목표로 삼은 위치와 방향의 JSON 객체</t>
+          <t>JSON object containing the target position and orientation for the recovery action.</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12735,12 +12735,12 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>행동 전 관측 데이터가 저장된 위치 URI</t>
+          <t>URI of the stored before state data.</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12787,12 +12787,12 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>행동 전 관측 파일의 무결성을 확인하는 SHA-256 해시</t>
+          <t>SHA-256 hash used to verify the integrity of the before state.</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12839,12 +12839,12 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>행동 후 관측 데이터가 저장된 위치 URI</t>
+          <t>URI of the stored after state data.</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12891,12 +12891,12 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>행동 후 관측 파일의 무결성을 확인하는 SHA-256 해시</t>
+          <t>SHA-256 hash used to verify the integrity of the after state.</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12943,12 +12943,12 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>RL 학습용 보상을 항목별로 기록한 JSON 객체</t>
+          <t>JSON object containing individual reward components for reinforcement learning.</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -12995,12 +12995,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>복구 결과를 safe, boundary 또는 critical로 구분한 코드</t>
+          <t>Outcome class for this record.</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -13047,12 +13047,12 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>복구 행동의 대기, 실행, 성공, 실패 또는 취소 상태 코드</t>
+          <t>Current execution status code.</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -13099,12 +13099,12 @@
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>해당 복구 행동이 에피소드의 마지막 단계인지 나타내는 값</t>
+          <t>Indicates whether this recovery action is the final step of the episode.</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -13151,12 +13151,12 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>업무, 단계 또는 복구 행동이 실제로 시작된 시각</t>
+          <t>Timestamp when the started event occurred.</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -13203,12 +13203,12 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>업무, 단계 또는 복구 행동이 완료된 시각</t>
+          <t>Timestamp when the completed event occurred.</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>
@@ -13255,12 +13255,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>해당 레코드가 데이터베이스에 생성된 시각</t>
+          <t>Timestamp when the created event occurred.</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>복구 에피소드에서 실제 실행한 행동, 전후 관측, 보상, 결과와 완료 상태를 순서대로 기록한다.</t>
+          <t>Records executed recovery actions, observations, rewards, outcomes, and completion status in sequence.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: persist structured task attempts
</commit_message>
<xml_diff>
--- a/docs/database/data_dictionary.xlsx
+++ b/docs/database/data_dictionary.xlsx
@@ -3479,7 +3479,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Job lifecycle status from pending and planning through execution, completion, failure, cancellation, or safety hold.</t>
+          <t>Job lifecycle status: queued, assigned, running, held, completed, failed, or cancelled.</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Job-step status: pending, queued, running, succeeded, failed, held, or cancelled.</t>
+          <t>Job-step status: pending, running, succeeded, failed, or cancelled.</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">

</xml_diff>